<commit_message>
add depth=4 model parameter
</commit_message>
<xml_diff>
--- a/group28/Group28_tables.xlsx
+++ b/group28/Group28_tables.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhangsw/Desktop/Leiden Univ/Semester3/Agentic_Large_Language_Models/Assignments/nanochat/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhangsw/Desktop/Leiden Univ/Semester3/Agentic_Large_Language_Models/AgenticLLMs_Assignment1_nanochat/group28/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8875926C-6558-1849-83E9-759B60FC8A1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4875F3C3-9862-9E4E-BFFD-9AAFBB0311B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5920" yWindow="1500" windowWidth="28100" windowHeight="17360" activeTab="1" xr2:uid="{81F75719-5437-3144-9CE3-AEA0A8A292AC}"/>
+    <workbookView xWindow="4100" yWindow="720" windowWidth="29480" windowHeight="19240" activeTab="1" xr2:uid="{81F75719-5437-3144-9CE3-AEA0A8A292AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Task 1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="108">
   <si>
     <t>Text Type
 (Text Length)</t>
@@ -84,10 +84,6 @@
   </si>
   <si>
     <t>Calculation</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Value</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -418,9 +414,6 @@
     <t>total_batch_size * num_iterations = 131,072 * 420</t>
   </si>
   <si>
-    <t>Σ(layers(12 * h * q * effective_seq)) = 12 * 1 * 128 * (512+2048)</t>
-  </si>
-  <si>
     <t>6 * num_matmul_params + atten_FLOPs</t>
   </si>
   <si>
@@ -464,6 +457,30 @@
   </si>
   <si>
     <t>embedding_width // head_dim = 128 // 128</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>depth=4</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>kv head</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>= attention head</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>-</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>depth=2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Σ(layers(12 * h * q * effective_seq)) = 12 * 1 * 128 * (512*(depth-1)+2048)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -474,8 +491,8 @@
   <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="181" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="185" formatCode="_(* #,##0.000000_);_(* \(#,##0.000000\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="_(* #,##0.000000_);_(* \(#,##0.000000\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -567,7 +584,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -595,6 +612,60 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -604,83 +675,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="185" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1041,7 +1049,7 @@
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="27" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2">
@@ -1055,7 +1063,7 @@
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="10"/>
+      <c r="A3" s="28"/>
       <c r="B3" s="6">
         <v>32768</v>
       </c>
@@ -1067,7 +1075,7 @@
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="27" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="2">
@@ -1081,7 +1089,7 @@
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="10"/>
+      <c r="A5" s="28"/>
       <c r="B5" s="6">
         <v>32768</v>
       </c>
@@ -1093,7 +1101,7 @@
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="27" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="2">
@@ -1107,7 +1115,7 @@
       </c>
     </row>
     <row r="7" spans="1:4">
-      <c r="A7" s="10"/>
+      <c r="A7" s="28"/>
       <c r="B7" s="6">
         <v>32768</v>
       </c>
@@ -1119,7 +1127,7 @@
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="29" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="3">
@@ -1133,7 +1141,7 @@
       </c>
     </row>
     <row r="9" spans="1:4">
-      <c r="A9" s="10"/>
+      <c r="A9" s="28"/>
       <c r="B9" s="6">
         <v>32768</v>
       </c>
@@ -1159,533 +1167,659 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93169463-092D-7846-950D-F7BAF9F35BA4}">
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="19"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="8"/>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" style="12" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" style="9" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="20">
-      <c r="A1" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="B1" s="26" t="s">
+      <c r="A1" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="27" t="s">
-        <v>10</v>
+      <c r="D1" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="E1" s="34" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="20">
       <c r="A2" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="15">
+        <v>2</v>
+      </c>
+      <c r="E2" s="15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="D2" s="22">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="D3" s="15">
+      <c r="B3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="11">
         <f>_xlfn.FLOOR.MATH((D2*64+128-1)/128)*128</f>
         <v>128</v>
       </c>
+      <c r="E3" s="11">
+        <f>_xlfn.FLOOR.MATH((E2*64+128-1)/128)*128</f>
+        <v>256</v>
+      </c>
       <c r="F3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="16"/>
-      <c r="B4" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="D4" s="15">
+      <c r="A4" s="29"/>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D4" s="11">
         <f>_xlfn.FLOOR.MATH(D3/128)</f>
         <v>1</v>
       </c>
+      <c r="E4" s="11">
+        <f>_xlfn.FLOOR.MATH(E3/128)</f>
+        <v>2</v>
+      </c>
       <c r="F4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="29"/>
+      <c r="B5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="32" t="s">
+        <v>104</v>
+      </c>
+      <c r="D5" s="11">
+        <f>D4</f>
+        <v>1</v>
+      </c>
+      <c r="E5" s="11">
+        <f>E4</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="29"/>
+      <c r="B6" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="16"/>
-      <c r="B5" s="14" t="s">
+      <c r="C6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="11">
+        <f>D37</f>
+        <v>12976170</v>
+      </c>
+      <c r="E6" s="11">
+        <f>E37</f>
+        <v>36700242</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="29"/>
+      <c r="B7" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C7" t="s">
         <v>48</v>
       </c>
-      <c r="D5" s="15">
-        <f>D36</f>
-        <v>12976170</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="16"/>
-      <c r="B6" s="14" t="s">
+      <c r="D7" s="11">
+        <f>D32+D33+D34+D35</f>
+        <v>4587532</v>
+      </c>
+      <c r="E7" s="11">
+        <f>E32+E33+E34+E35</f>
+        <v>11534384</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="29"/>
+      <c r="B8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="11">
+        <f>D7+24</f>
+        <v>4587556</v>
+      </c>
+      <c r="E8" s="11">
+        <f>E7+24</f>
+        <v>11534408</v>
+      </c>
+      <c r="F8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C9" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="D6" s="15">
-        <f>D31+D32+D33+D34</f>
-        <v>4587532</v>
-      </c>
-      <c r="E6">
-        <v>4587532</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="16"/>
-      <c r="B7" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C7" s="14" t="s">
+      <c r="D9" s="17">
+        <v>12</v>
+      </c>
+      <c r="E9" s="17">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="29"/>
+      <c r="B10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" t="s">
+        <v>88</v>
+      </c>
+      <c r="D10" s="11">
+        <f>D7*D9</f>
+        <v>55050384</v>
+      </c>
+      <c r="E10" s="11">
+        <f>E7*E9</f>
+        <v>138412608</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="29"/>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" t="s">
+        <v>89</v>
+      </c>
+      <c r="D11" s="11">
+        <f>D18*D19</f>
+        <v>55050240</v>
+      </c>
+      <c r="E11" s="11">
+        <f>E18*E19</f>
+        <v>138412032</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="31"/>
+      <c r="B12" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="13">
+        <v>2048</v>
+      </c>
+      <c r="E12" s="13">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="19" customHeight="1">
+      <c r="A13" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" t="s">
         <v>61</v>
       </c>
-      <c r="D7" s="15">
-        <f>D6+24</f>
-        <v>4587556</v>
-      </c>
-      <c r="F7" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" s="24">
-        <v>12</v>
-      </c>
-      <c r="E8">
-        <v>20</v>
-      </c>
-      <c r="F8" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="16"/>
-      <c r="B9" s="14" t="s">
+      <c r="C13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D13" s="11">
+        <f>12*1*D3*(512*(D2-1)+D12)</f>
+        <v>3932160</v>
+      </c>
+      <c r="E13" s="11">
+        <f>12*1*E3*(512*(E2-1)+E12)</f>
+        <v>11010048</v>
+      </c>
+      <c r="F13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="29"/>
+      <c r="B14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" t="s">
+        <v>90</v>
+      </c>
+      <c r="D14" s="11">
+        <f>6*D8+D13</f>
+        <v>31457496</v>
+      </c>
+      <c r="E14" s="11">
+        <f>6*E8+E13</f>
+        <v>80216496</v>
+      </c>
+      <c r="F14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="31"/>
+      <c r="B15" t="s">
+        <v>97</v>
+      </c>
+      <c r="C15" t="s">
+        <v>98</v>
+      </c>
+      <c r="D15" s="26">
+        <f>D14*D11</f>
+        <v>1731742704599040</v>
+      </c>
+      <c r="E15" s="26">
+        <f>E14*E11</f>
+        <v>1.1102928211279872E+16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="27" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="C9" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="D9" s="15">
-        <f>D6*D8</f>
-        <v>55050384</v>
-      </c>
-      <c r="E9" s="15">
-        <f>E6*E8</f>
-        <v>91750640</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" s="16"/>
-      <c r="B10" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="D10" s="15">
-        <f>D17*D18</f>
-        <v>55050240</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="18"/>
-      <c r="B11" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="20">
-        <v>2048</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="19" customHeight="1">
-      <c r="A12" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="D12" s="15">
-        <f>12*1*D3*(512+D11)</f>
-        <v>3932160</v>
-      </c>
-      <c r="F12" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" s="16"/>
-      <c r="B13" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="D13" s="15">
-        <f>6*D7+D12</f>
-        <v>31457496</v>
-      </c>
-      <c r="F13" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="18"/>
-      <c r="B14" s="28" t="s">
-        <v>99</v>
-      </c>
-      <c r="C14" s="28" t="s">
-        <v>100</v>
-      </c>
-      <c r="D14" s="36">
-        <f>D13*D10</f>
-        <v>1731742704599040</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="B15" s="23" t="s">
+      <c r="D16" s="33" t="s">
+        <v>105</v>
+      </c>
+      <c r="E16" s="33" t="s">
+        <v>105</v>
+      </c>
+      <c r="F16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="31"/>
+      <c r="B17" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C15" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="D15" s="24">
-        <f>D21/0.28/SQRT(D17/D16)*D9</f>
-        <v>1321210788.8681142</v>
-      </c>
-      <c r="F15" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="18"/>
-      <c r="B16" s="19" t="s">
+      <c r="C17" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="C16" s="25" t="s">
-        <v>71</v>
-      </c>
-      <c r="D16" s="20">
+      <c r="D17" s="13">
         <f>2^19</f>
         <v>524288</v>
       </c>
-      <c r="F16" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="19" customHeight="1">
-      <c r="A17" s="9" t="s">
+      <c r="E17" s="13">
+        <f>2^19</f>
+        <v>524288</v>
+      </c>
+      <c r="F17" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="19" customHeight="1">
+      <c r="A18" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="B18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>95</v>
+      </c>
+      <c r="D18" s="11">
+        <v>131072</v>
+      </c>
+      <c r="E18" s="11">
+        <v>262144</v>
+      </c>
+      <c r="F18" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="29"/>
+      <c r="B19" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="11">
+        <f>_xlfn.FLOOR.MATH(D10/D18)</f>
+        <v>420</v>
+      </c>
+      <c r="E19" s="11">
+        <f>_xlfn.FLOOR.MATH(E10/E18)</f>
+        <v>528</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="27" t="s">
         <v>77</v>
       </c>
-      <c r="B17" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="D17" s="15">
-        <v>131072</v>
-      </c>
-      <c r="F17" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" s="16"/>
-      <c r="B18" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C18" s="14" t="s">
+      <c r="B20" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="D18" s="15">
-        <f>_xlfn.FLOOR.MATH(D9/D17)</f>
-        <v>420</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="B19" s="23" t="s">
+      <c r="D20" s="20">
+        <f>SQRT(D18/D17)</f>
+        <v>0.5</v>
+      </c>
+      <c r="E20" s="20">
+        <f>SQRT(E18/E17)</f>
+        <v>0.70710678118654757</v>
+      </c>
+      <c r="F20" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="29"/>
+      <c r="B21" t="s">
         <v>54</v>
       </c>
-      <c r="C19" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="D19" s="29">
-        <f>SQRT(D17/D16)</f>
-        <v>0.5</v>
-      </c>
-      <c r="F19" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="16"/>
-      <c r="B20" s="14" t="s">
+      <c r="C21" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="D20" s="35">
+      <c r="D21" s="25">
         <f>(D3/768)^(-1/2)</f>
         <v>2.4494897427831779</v>
       </c>
-      <c r="F20" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" s="16"/>
-      <c r="B21" s="28" t="s">
-        <v>101</v>
-      </c>
-      <c r="C21" s="30" t="s">
-        <v>98</v>
-      </c>
-      <c r="D21" s="35">
+      <c r="E21" s="25">
+        <f>(E3/768)^(-1/2)</f>
+        <v>1.7320508075688774</v>
+      </c>
+      <c r="F21" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="29"/>
+      <c r="B22" t="s">
+        <v>99</v>
+      </c>
+      <c r="C22" t="s">
+        <v>96</v>
+      </c>
+      <c r="D22" s="25">
         <v>3.360004</v>
       </c>
-      <c r="E21" s="37"/>
-      <c r="F21" t="s">
+      <c r="E22">
+        <v>1.8899030000000001</v>
+      </c>
+      <c r="F22" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="29"/>
+      <c r="B23" t="s">
+        <v>56</v>
+      </c>
+      <c r="C23" t="s">
+        <v>57</v>
+      </c>
+      <c r="D23" s="11">
+        <v>16</v>
+      </c>
+      <c r="E23" s="11">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="29"/>
+      <c r="B24" t="s">
+        <v>80</v>
+      </c>
+      <c r="C24" t="s">
+        <v>82</v>
+      </c>
+      <c r="D24" s="11">
+        <v>1</v>
+      </c>
+      <c r="E24" s="11">
+        <v>1</v>
+      </c>
+      <c r="F24" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" s="31"/>
+      <c r="B25" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="D25" s="13">
+        <f>D18/(D23*D12*D24)</f>
+        <v>4</v>
+      </c>
+      <c r="E25" s="13">
+        <f>E18/(E23*E12*E24)</f>
+        <v>8</v>
+      </c>
+      <c r="F25" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="B28" s="21" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="B29" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C29" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="E29" s="24" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="A22" s="16"/>
-      <c r="B22" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="C22" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="D22" s="15">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6">
-      <c r="A23" s="16"/>
-      <c r="B23" s="28" t="s">
-        <v>81</v>
-      </c>
-      <c r="C23" s="30" t="s">
-        <v>83</v>
-      </c>
-      <c r="D23" s="15">
-        <v>1</v>
-      </c>
-      <c r="F23" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24" s="18"/>
-      <c r="B24" s="19" t="s">
+      <c r="F29" s="22" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="B30" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C30" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="19" t="s">
-        <v>93</v>
-      </c>
-      <c r="D24" s="20">
-        <f>D17/(D22*D11*D23)</f>
-        <v>4</v>
-      </c>
-      <c r="F24" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="B27" s="31" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="B28" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="C28" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="D28" s="33" t="s">
-        <v>10</v>
-      </c>
-      <c r="E28" s="32" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6">
-      <c r="B29" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="C29" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="D29" s="24">
+      <c r="D30" s="17">
         <f>32768*D3</f>
         <v>4194304</v>
       </c>
-      <c r="E29" s="23" t="s">
+      <c r="E30" s="17">
+        <f>32768*E3</f>
+        <v>8388608</v>
+      </c>
+      <c r="F30" s="16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="B31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C31" t="s">
+        <v>25</v>
+      </c>
+      <c r="D31" s="11">
+        <f>_xlfn.FLOOR.MATH((D2+1)/2)*32768*D3</f>
+        <v>4194304</v>
+      </c>
+      <c r="E31" s="11">
+        <f>_xlfn.FLOOR.MATH((E2+1)/2)*32768*E3</f>
+        <v>16777216</v>
+      </c>
+      <c r="F31" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
-      <c r="B30" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C30" s="14" t="s">
+    <row r="32" spans="1:6">
+      <c r="B32" t="s">
         <v>26</v>
       </c>
-      <c r="D30" s="15">
-        <f>1*32768*D3</f>
-        <v>4194304</v>
-      </c>
-      <c r="E30" s="14" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6">
-      <c r="B31" s="14" t="s">
+      <c r="C32" t="s">
         <v>27</v>
       </c>
-      <c r="C31" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="D31" s="15">
+      <c r="D32" s="11">
         <f>32768*D3</f>
         <v>4194304</v>
       </c>
-      <c r="E31" s="14" t="s">
+      <c r="E32" s="11">
+        <f>32768*E3</f>
+        <v>8388608</v>
+      </c>
+      <c r="F32" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6">
+      <c r="B33" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33" t="s">
+        <v>35</v>
+      </c>
+      <c r="D33" s="11">
+        <f>(D3*(D4+2*D5)*128+D3*D3)*D2</f>
+        <v>131072</v>
+      </c>
+      <c r="E33" s="11">
+        <f>(E3*(E4+2*E5)*128+E3*E3)*E2</f>
+        <v>1048576</v>
+      </c>
+      <c r="F33" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
-      <c r="B32" s="14" t="s">
+    <row r="34" spans="2:6">
+      <c r="B34" t="s">
+        <v>31</v>
+      </c>
+      <c r="C34" t="s">
+        <v>32</v>
+      </c>
+      <c r="D34" s="11">
+        <f>_xlfn.FLOOR.MATH((D2+1)/2)*12*D5</f>
+        <v>12</v>
+      </c>
+      <c r="E34" s="11">
+        <f>_xlfn.FLOOR.MATH((E2+1)/2)*12*E5</f>
+        <v>48</v>
+      </c>
+      <c r="F34" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6">
+      <c r="B35" t="s">
         <v>29</v>
       </c>
-      <c r="C32" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="D32" s="15">
-        <f>(D3*3*128+D3*D3)*D2</f>
-        <v>131072</v>
-      </c>
-      <c r="E32" s="14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="33" spans="2:5">
-      <c r="B33" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C33" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="D33" s="15">
-        <f>_xlfn.FLOOR.MATH((2+1)/2)*12*1</f>
-        <v>12</v>
-      </c>
-      <c r="E33" s="14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="34" spans="2:5">
-      <c r="B34" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C34" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="D34" s="15">
+      <c r="C35" t="s">
+        <v>34</v>
+      </c>
+      <c r="D35" s="11">
         <f>D3*4*D3*2*D2</f>
         <v>262144</v>
       </c>
-      <c r="E34" s="14" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="35" spans="2:5">
-      <c r="B35" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="C35" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="D35" s="20">
+      <c r="E35" s="11">
+        <f>E3*4*E3*2*E2</f>
+        <v>2097152</v>
+      </c>
+      <c r="F35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6">
+      <c r="B36" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D36" s="13">
         <f>D2+D2+24+1+1</f>
         <v>30</v>
       </c>
-      <c r="E35" s="19" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="36" spans="2:5">
-      <c r="B36" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="C36" s="34"/>
-      <c r="D36" s="33">
-        <f>SUM(D29:D35)</f>
+      <c r="E36" s="13">
+        <v>34</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6">
+      <c r="B37" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" s="30"/>
+      <c r="D37" s="23">
+        <f>SUM(D30:D36)</f>
         <v>12976170</v>
       </c>
-      <c r="E36" s="21"/>
+      <c r="E37" s="23">
+        <f>SUM(E30:E36)</f>
+        <v>36700242</v>
+      </c>
+      <c r="F37" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="A3:A7"/>
-    <mergeCell ref="A8:A11"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A19:A24"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="A3:A8"/>
+    <mergeCell ref="A9:A12"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A20:A25"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A13:A15"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update tables in report
</commit_message>
<xml_diff>
--- a/group28/Group28_tables.xlsx
+++ b/group28/Group28_tables.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhangsw/Desktop/Leiden Univ/Semester3/Agentic_Large_Language_Models/AgenticLLMs_Assignment1_nanochat/group28/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4875F3C3-9862-9E4E-BFFD-9AAFBB0311B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FF8CA01-F3F6-3D4A-9F20-48668C968811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4100" yWindow="720" windowWidth="29480" windowHeight="19240" activeTab="1" xr2:uid="{81F75719-5437-3144-9CE3-AEA0A8A292AC}"/>
+    <workbookView xWindow="4120" yWindow="500" windowWidth="26900" windowHeight="18160" xr2:uid="{81F75719-5437-3144-9CE3-AEA0A8A292AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Task 1" sheetId="1" r:id="rId1"/>
     <sheet name="Task 2 Model" sheetId="2" r:id="rId2"/>
+    <sheet name="Task 3 Loss Masking" sheetId="3" r:id="rId3"/>
+    <sheet name="Task 3 Data Analysis" sheetId="4" r:id="rId4"/>
+    <sheet name="Task 3 Benchmark Score" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="145">
   <si>
     <t>Text Type
 (Text Length)</t>
@@ -483,6 +486,145 @@
     <t>Σ(layers(12 * h * q * effective_seq)) = 12 * 1 * 128 * (512*(depth-1)+2048)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
+  <si>
+    <t>Input token</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Target token</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Masked target</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;|bos|&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Compute</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>+</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;|user_end|&gt;</t>
+  </si>
+  <si>
+    <t>&lt;|assistant_start|&gt;</t>
+  </si>
+  <si>
+    <t>&lt;|assistant_end|&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>from tokenizer.render_conversation()</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;|user_start|&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dataset</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GSM8K</t>
+  </si>
+  <si>
+    <t>Stage</t>
+  </si>
+  <si>
+    <t>Stage</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mid-training</t>
+  </si>
+  <si>
+    <t>Mid-training</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SFT</t>
+  </si>
+  <si>
+    <t>SFT</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Train size</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Test size</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Total size</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Smol-SmolTalk</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MMLU auxiliary train</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>dev</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>valid</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Repetition</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Effective size</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Model tag</t>
+  </si>
+  <si>
+    <t>Step</t>
+  </si>
+  <si>
+    <t>Base</t>
+  </si>
+  <si>
+    <t>depth2_eval50</t>
+  </si>
+  <si>
+    <t>depth2_midtrain</t>
+  </si>
+  <si>
+    <t>depth2_sft</t>
+  </si>
+  <si>
+    <t>ARC-Easy
+(2376)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ARC-Challenge
+(1172)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GSM8K
+(1319)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -494,7 +636,7 @@
     <numFmt numFmtId="177" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="178" formatCode="_(* #,##0.000000_);_(* \(#,##0.000000\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -528,6 +670,24 @@
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Menlo Regular"/>
     </font>
   </fonts>
   <fills count="2">
@@ -584,7 +744,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -666,6 +826,15 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -681,13 +850,52 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1035,21 +1243,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="40">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="46" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="30" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2">
@@ -1063,7 +1271,7 @@
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="28"/>
+      <c r="A3" s="31"/>
       <c r="B3" s="6">
         <v>32768</v>
       </c>
@@ -1075,7 +1283,7 @@
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="30" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="2">
@@ -1089,7 +1297,7 @@
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="28"/>
+      <c r="A5" s="31"/>
       <c r="B5" s="6">
         <v>32768</v>
       </c>
@@ -1101,7 +1309,7 @@
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="30" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="2">
@@ -1115,7 +1323,7 @@
       </c>
     </row>
     <row r="7" spans="1:4">
-      <c r="A7" s="28"/>
+      <c r="A7" s="31"/>
       <c r="B7" s="6">
         <v>32768</v>
       </c>
@@ -1127,7 +1335,7 @@
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="32" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="3">
@@ -1141,7 +1349,7 @@
       </c>
     </row>
     <row r="9" spans="1:4">
-      <c r="A9" s="28"/>
+      <c r="A9" s="31"/>
       <c r="B9" s="6">
         <v>32768</v>
       </c>
@@ -1187,10 +1395,10 @@
       <c r="C1" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="34" t="s">
+      <c r="D1" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="E1" s="34" t="s">
+      <c r="E1" s="29" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1212,7 +1420,7 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="32" t="s">
         <v>64</v>
       </c>
       <c r="B3" t="s">
@@ -1234,7 +1442,7 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="29"/>
+      <c r="A4" s="32"/>
       <c r="B4" t="s">
         <v>11</v>
       </c>
@@ -1254,11 +1462,11 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="29"/>
+      <c r="A5" s="32"/>
       <c r="B5" t="s">
         <v>103</v>
       </c>
-      <c r="C5" s="32" t="s">
+      <c r="C5" s="27" t="s">
         <v>104</v>
       </c>
       <c r="D5" s="11">
@@ -1271,7 +1479,7 @@
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="29"/>
+      <c r="A6" s="32"/>
       <c r="B6" t="s">
         <v>14</v>
       </c>
@@ -1288,7 +1496,7 @@
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="29"/>
+      <c r="A7" s="32"/>
       <c r="B7" t="s">
         <v>15</v>
       </c>
@@ -1305,7 +1513,7 @@
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="29"/>
+      <c r="A8" s="32"/>
       <c r="B8" t="s">
         <v>59</v>
       </c>
@@ -1325,7 +1533,7 @@
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="27" t="s">
+      <c r="A9" s="30" t="s">
         <v>73</v>
       </c>
       <c r="B9" s="16" t="s">
@@ -1345,7 +1553,7 @@
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="29"/>
+      <c r="A10" s="32"/>
       <c r="B10" t="s">
         <v>66</v>
       </c>
@@ -1362,7 +1570,7 @@
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="29"/>
+      <c r="A11" s="32"/>
       <c r="B11" t="s">
         <v>18</v>
       </c>
@@ -1379,7 +1587,7 @@
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="31"/>
+      <c r="A12" s="34"/>
       <c r="B12" s="12" t="s">
         <v>46</v>
       </c>
@@ -1394,7 +1602,7 @@
       </c>
     </row>
     <row r="13" spans="1:6" ht="19" customHeight="1">
-      <c r="A13" s="27" t="s">
+      <c r="A13" s="30" t="s">
         <v>74</v>
       </c>
       <c r="B13" t="s">
@@ -1416,7 +1624,7 @@
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="29"/>
+      <c r="A14" s="32"/>
       <c r="B14" t="s">
         <v>45</v>
       </c>
@@ -1436,7 +1644,7 @@
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="31"/>
+      <c r="A15" s="34"/>
       <c r="B15" t="s">
         <v>97</v>
       </c>
@@ -1453,7 +1661,7 @@
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="30" t="s">
         <v>75</v>
       </c>
       <c r="B16" s="16" t="s">
@@ -1462,10 +1670,10 @@
       <c r="C16" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="D16" s="33" t="s">
+      <c r="D16" s="28" t="s">
         <v>105</v>
       </c>
-      <c r="E16" s="33" t="s">
+      <c r="E16" s="28" t="s">
         <v>105</v>
       </c>
       <c r="F16" t="s">
@@ -1473,7 +1681,7 @@
       </c>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="31"/>
+      <c r="A17" s="34"/>
       <c r="B17" s="12" t="s">
         <v>69</v>
       </c>
@@ -1493,7 +1701,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="19" customHeight="1">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="30" t="s">
         <v>76</v>
       </c>
       <c r="B18" t="s">
@@ -1513,7 +1721,7 @@
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="29"/>
+      <c r="A19" s="32"/>
       <c r="B19" t="s">
         <v>19</v>
       </c>
@@ -1530,7 +1738,7 @@
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="27" t="s">
+      <c r="A20" s="30" t="s">
         <v>77</v>
       </c>
       <c r="B20" s="16" t="s">
@@ -1552,7 +1760,7 @@
       </c>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="29"/>
+      <c r="A21" s="32"/>
       <c r="B21" t="s">
         <v>54</v>
       </c>
@@ -1572,7 +1780,7 @@
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="29"/>
+      <c r="A22" s="32"/>
       <c r="B22" t="s">
         <v>99</v>
       </c>
@@ -1590,7 +1798,7 @@
       </c>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="29"/>
+      <c r="A23" s="32"/>
       <c r="B23" t="s">
         <v>56</v>
       </c>
@@ -1605,7 +1813,7 @@
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="29"/>
+      <c r="A24" s="32"/>
       <c r="B24" t="s">
         <v>80</v>
       </c>
@@ -1623,7 +1831,7 @@
       </c>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="31"/>
+      <c r="A25" s="34"/>
       <c r="B25" s="12" t="s">
         <v>20</v>
       </c>
@@ -1797,10 +2005,10 @@
       </c>
     </row>
     <row r="37" spans="2:6">
-      <c r="B37" s="30" t="s">
+      <c r="B37" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="C37" s="30"/>
+      <c r="C37" s="33"/>
       <c r="D37" s="23">
         <f>SUM(D30:D36)</f>
         <v>12976170</v>
@@ -1825,4 +2033,364 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EDA6DF4-0FA4-1D4F-B91E-7CAE46A734FF}">
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="2" width="21.5703125" style="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" style="36" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="10.7109375" style="36"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="35" customFormat="1" ht="16">
+      <c r="A1" s="38" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1" s="38" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="39" t="s">
+        <v>111</v>
+      </c>
+      <c r="B2" s="39" t="s">
+        <v>118</v>
+      </c>
+      <c r="C2" s="39">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="40" t="s">
+        <v>118</v>
+      </c>
+      <c r="B3" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="C3" s="40">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="B4" s="40">
+        <v>1</v>
+      </c>
+      <c r="C4" s="40">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="40">
+        <v>1</v>
+      </c>
+      <c r="B5" s="40" t="s">
+        <v>113</v>
+      </c>
+      <c r="C5" s="40">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="40" t="s">
+        <v>113</v>
+      </c>
+      <c r="B6" s="40">
+        <v>1</v>
+      </c>
+      <c r="C6" s="40">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="40">
+        <v>1</v>
+      </c>
+      <c r="B7" s="40" t="s">
+        <v>114</v>
+      </c>
+      <c r="C7" s="40">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="40" t="s">
+        <v>114</v>
+      </c>
+      <c r="B8" s="40" t="s">
+        <v>115</v>
+      </c>
+      <c r="C8" s="40">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="40" t="s">
+        <v>115</v>
+      </c>
+      <c r="B9" s="40">
+        <v>2</v>
+      </c>
+      <c r="C9" s="40">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="41">
+        <v>2</v>
+      </c>
+      <c r="B10" s="41" t="s">
+        <v>116</v>
+      </c>
+      <c r="C10" s="41" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="37" t="s">
+        <v>117</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{778F4F05-A398-0346-B331-564F10C2C771}">
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="19"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.7109375" style="4"/>
+    <col min="5" max="5" width="12.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="10.7109375" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="B1" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" s="24" t="s">
+        <v>127</v>
+      </c>
+      <c r="D1" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E1" s="24" t="s">
+        <v>135</v>
+      </c>
+      <c r="F1" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="G1" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" s="42">
+        <v>99842</v>
+      </c>
+      <c r="D2" s="42">
+        <v>3</v>
+      </c>
+      <c r="E2" s="42">
+        <f>C2*D2</f>
+        <v>299526</v>
+      </c>
+      <c r="F2" s="42">
+        <v>14042</v>
+      </c>
+      <c r="G2" s="42">
+        <f>C2+F2+H2+I2</f>
+        <v>115700</v>
+      </c>
+      <c r="H2" s="4">
+        <v>285</v>
+      </c>
+      <c r="I2" s="4">
+        <v>1531</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="43" t="s">
+        <v>124</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" s="44">
+        <v>7473</v>
+      </c>
+      <c r="D3" s="44">
+        <v>4</v>
+      </c>
+      <c r="E3" s="44">
+        <f t="shared" ref="E3:E4" si="0">C3*D3</f>
+        <v>29892</v>
+      </c>
+      <c r="F3" s="44">
+        <v>1319</v>
+      </c>
+      <c r="G3" s="44">
+        <f>C3+F3</f>
+        <v>8792</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C4" s="45">
+        <v>460341</v>
+      </c>
+      <c r="D4" s="45">
+        <v>1</v>
+      </c>
+      <c r="E4" s="45">
+        <f t="shared" si="0"/>
+        <v>460341</v>
+      </c>
+      <c r="F4" s="45">
+        <v>24229</v>
+      </c>
+      <c r="G4" s="45">
+        <v>484570</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{574B76E6-61C4-B449-A074-3BDA90F1367C}">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="19"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" customWidth="1"/>
+    <col min="3" max="3" width="5.7109375" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="40">
+      <c r="A1" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="B1" s="24" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1" s="24" t="s">
+        <v>137</v>
+      </c>
+      <c r="D1" s="46" t="s">
+        <v>142</v>
+      </c>
+      <c r="E1" s="46" t="s">
+        <v>143</v>
+      </c>
+      <c r="F1" s="46" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="43" t="s">
+        <v>138</v>
+      </c>
+      <c r="B2" s="43" t="s">
+        <v>139</v>
+      </c>
+      <c r="C2" s="43">
+        <v>420</v>
+      </c>
+      <c r="D2" s="47">
+        <v>0.2487</v>
+      </c>
+      <c r="E2" s="47">
+        <v>0.23630000000000001</v>
+      </c>
+      <c r="F2" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" s="43">
+        <v>928</v>
+      </c>
+      <c r="D3" s="47">
+        <v>0.2576</v>
+      </c>
+      <c r="E3" s="47">
+        <v>0.28160000000000002</v>
+      </c>
+      <c r="F3" s="47">
+        <v>9.9000000000000008E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="C4" s="5">
+        <v>2868</v>
+      </c>
+      <c r="D4" s="48">
+        <v>0.25130000000000002</v>
+      </c>
+      <c r="E4" s="48">
+        <v>0.2329</v>
+      </c>
+      <c r="F4" s="50">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add absolute corret number and the total number of test split
</commit_message>
<xml_diff>
--- a/group28/Group28_tables.xlsx
+++ b/group28/Group28_tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhangsw/Desktop/Leiden Univ/Semester3/Agentic_Large_Language_Models/AgenticLLMs_Assignment1_nanochat/group28/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FF8CA01-F3F6-3D4A-9F20-48668C968811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F20B42D6-2B02-A940-96FA-A232C342719B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4120" yWindow="500" windowWidth="26900" windowHeight="18160" xr2:uid="{81F75719-5437-3144-9CE3-AEA0A8A292AC}"/>
+    <workbookView xWindow="4480" yWindow="500" windowWidth="26900" windowHeight="18160" activeTab="4" xr2:uid="{81F75719-5437-3144-9CE3-AEA0A8A292AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Task 1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="153">
   <si>
     <t>Text Type
 (Text Length)</t>
@@ -611,18 +611,42 @@
     <t>depth2_sft</t>
   </si>
   <si>
+    <t>591 (24.87%)</t>
+  </si>
+  <si>
+    <t>277 (23.63%)</t>
+  </si>
+  <si>
+    <t>0 (0.0%)</t>
+  </si>
+  <si>
+    <t>612 (25.76%)</t>
+  </si>
+  <si>
+    <t>330 (28.16%)</t>
+  </si>
+  <si>
+    <t>13 (0.99%)</t>
+  </si>
+  <si>
+    <t>597 (25.13%)</t>
+  </si>
+  <si>
+    <t>273 (23.29%)</t>
+  </si>
+  <si>
     <t>ARC-Easy
-(2376)</t>
+(N=2376)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>ARC-Challenge
-(1172)</t>
+(N=1172)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>GSM8K
-(1319)</t>
+(N=1319)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -744,7 +768,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -835,6 +859,48 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -849,54 +915,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1243,21 +1261,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="40">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="46" t="s">
+      <c r="C1" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="46" t="s">
+      <c r="D1" s="39" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="44" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2">
@@ -1271,7 +1289,7 @@
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="31"/>
+      <c r="A3" s="45"/>
       <c r="B3" s="6">
         <v>32768</v>
       </c>
@@ -1283,7 +1301,7 @@
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="44" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="2">
@@ -1297,7 +1315,7 @@
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="31"/>
+      <c r="A5" s="45"/>
       <c r="B5" s="6">
         <v>32768</v>
       </c>
@@ -1309,7 +1327,7 @@
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="44" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="2">
@@ -1323,7 +1341,7 @@
       </c>
     </row>
     <row r="7" spans="1:4">
-      <c r="A7" s="31"/>
+      <c r="A7" s="45"/>
       <c r="B7" s="6">
         <v>32768</v>
       </c>
@@ -1335,7 +1353,7 @@
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="46" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="3">
@@ -1349,7 +1367,7 @@
       </c>
     </row>
     <row r="9" spans="1:4">
-      <c r="A9" s="31"/>
+      <c r="A9" s="45"/>
       <c r="B9" s="6">
         <v>32768</v>
       </c>
@@ -1420,7 +1438,7 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="46" t="s">
         <v>64</v>
       </c>
       <c r="B3" t="s">
@@ -1442,7 +1460,7 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="32"/>
+      <c r="A4" s="46"/>
       <c r="B4" t="s">
         <v>11</v>
       </c>
@@ -1462,7 +1480,7 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="32"/>
+      <c r="A5" s="46"/>
       <c r="B5" t="s">
         <v>103</v>
       </c>
@@ -1479,7 +1497,7 @@
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="32"/>
+      <c r="A6" s="46"/>
       <c r="B6" t="s">
         <v>14</v>
       </c>
@@ -1496,7 +1514,7 @@
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="32"/>
+      <c r="A7" s="46"/>
       <c r="B7" t="s">
         <v>15</v>
       </c>
@@ -1513,7 +1531,7 @@
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="32"/>
+      <c r="A8" s="46"/>
       <c r="B8" t="s">
         <v>59</v>
       </c>
@@ -1533,7 +1551,7 @@
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="30" t="s">
+      <c r="A9" s="44" t="s">
         <v>73</v>
       </c>
       <c r="B9" s="16" t="s">
@@ -1553,7 +1571,7 @@
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="32"/>
+      <c r="A10" s="46"/>
       <c r="B10" t="s">
         <v>66</v>
       </c>
@@ -1570,7 +1588,7 @@
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="32"/>
+      <c r="A11" s="46"/>
       <c r="B11" t="s">
         <v>18</v>
       </c>
@@ -1587,7 +1605,7 @@
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="34"/>
+      <c r="A12" s="48"/>
       <c r="B12" s="12" t="s">
         <v>46</v>
       </c>
@@ -1602,7 +1620,7 @@
       </c>
     </row>
     <row r="13" spans="1:6" ht="19" customHeight="1">
-      <c r="A13" s="30" t="s">
+      <c r="A13" s="44" t="s">
         <v>74</v>
       </c>
       <c r="B13" t="s">
@@ -1624,7 +1642,7 @@
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="32"/>
+      <c r="A14" s="46"/>
       <c r="B14" t="s">
         <v>45</v>
       </c>
@@ -1644,7 +1662,7 @@
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="34"/>
+      <c r="A15" s="48"/>
       <c r="B15" t="s">
         <v>97</v>
       </c>
@@ -1661,7 +1679,7 @@
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="44" t="s">
         <v>75</v>
       </c>
       <c r="B16" s="16" t="s">
@@ -1681,7 +1699,7 @@
       </c>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="34"/>
+      <c r="A17" s="48"/>
       <c r="B17" s="12" t="s">
         <v>69</v>
       </c>
@@ -1701,7 +1719,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="19" customHeight="1">
-      <c r="A18" s="30" t="s">
+      <c r="A18" s="44" t="s">
         <v>76</v>
       </c>
       <c r="B18" t="s">
@@ -1721,7 +1739,7 @@
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="32"/>
+      <c r="A19" s="46"/>
       <c r="B19" t="s">
         <v>19</v>
       </c>
@@ -1738,7 +1756,7 @@
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="30" t="s">
+      <c r="A20" s="44" t="s">
         <v>77</v>
       </c>
       <c r="B20" s="16" t="s">
@@ -1760,7 +1778,7 @@
       </c>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="32"/>
+      <c r="A21" s="46"/>
       <c r="B21" t="s">
         <v>54</v>
       </c>
@@ -1780,7 +1798,7 @@
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="32"/>
+      <c r="A22" s="46"/>
       <c r="B22" t="s">
         <v>99</v>
       </c>
@@ -1798,7 +1816,7 @@
       </c>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="32"/>
+      <c r="A23" s="46"/>
       <c r="B23" t="s">
         <v>56</v>
       </c>
@@ -1813,7 +1831,7 @@
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="32"/>
+      <c r="A24" s="46"/>
       <c r="B24" t="s">
         <v>80</v>
       </c>
@@ -1831,7 +1849,7 @@
       </c>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="34"/>
+      <c r="A25" s="48"/>
       <c r="B25" s="12" t="s">
         <v>20</v>
       </c>
@@ -2005,10 +2023,10 @@
       </c>
     </row>
     <row r="37" spans="2:6">
-      <c r="B37" s="33" t="s">
+      <c r="B37" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="C37" s="33"/>
+      <c r="C37" s="47"/>
       <c r="D37" s="23">
         <f>SUM(D30:D36)</f>
         <v>12976170</v>
@@ -2040,123 +2058,123 @@
   <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="21.5703125" style="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" style="36" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="10.7109375" style="36"/>
+    <col min="1" max="2" width="21.5703125" style="31" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" style="31" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="10.7109375" style="31"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="35" customFormat="1" ht="16">
-      <c r="A1" s="38" t="s">
+    <row r="1" spans="1:3" s="30" customFormat="1" ht="16">
+      <c r="A1" s="33" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="38" t="s">
+      <c r="B1" s="33" t="s">
         <v>109</v>
       </c>
-      <c r="C1" s="38" t="s">
+      <c r="C1" s="33" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="34" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="34" t="s">
         <v>118</v>
       </c>
-      <c r="C2" s="39">
+      <c r="C2" s="34">
         <v>-1</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="31" t="s">
         <v>118</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="C3" s="40">
+      <c r="C3" s="31">
         <v>-1</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="40">
+      <c r="B4" s="31">
         <v>1</v>
       </c>
-      <c r="C4" s="40">
+      <c r="C4" s="31">
         <v>-1</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="40">
+      <c r="A5" s="31">
         <v>1</v>
       </c>
-      <c r="B5" s="40" t="s">
+      <c r="B5" s="31" t="s">
         <v>113</v>
       </c>
-      <c r="C5" s="40">
+      <c r="C5" s="31">
         <v>-1</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="40" t="s">
+      <c r="A6" s="31" t="s">
         <v>113</v>
       </c>
-      <c r="B6" s="40">
+      <c r="B6" s="31">
         <v>1</v>
       </c>
-      <c r="C6" s="40">
+      <c r="C6" s="31">
         <v>-1</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="40">
+      <c r="A7" s="31">
         <v>1</v>
       </c>
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="31" t="s">
         <v>114</v>
       </c>
-      <c r="C7" s="40">
+      <c r="C7" s="31">
         <v>-1</v>
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" s="40" t="s">
+      <c r="A8" s="31" t="s">
         <v>114</v>
       </c>
-      <c r="B8" s="40" t="s">
+      <c r="B8" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="C8" s="40">
+      <c r="C8" s="31">
         <v>-1</v>
       </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" s="40" t="s">
+      <c r="A9" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="B9" s="40">
+      <c r="B9" s="31">
         <v>2</v>
       </c>
-      <c r="C9" s="40">
+      <c r="C9" s="31">
         <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="A10" s="41">
+      <c r="A10" s="35">
         <v>2</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="35" t="s">
         <v>116</v>
       </c>
-      <c r="C10" s="41" t="s">
+      <c r="C10" s="35" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="16" spans="1:3">
-      <c r="A16" s="37" t="s">
+      <c r="A16" s="32" t="s">
         <v>117</v>
       </c>
     </row>
@@ -2215,20 +2233,20 @@
       <c r="B2" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="42">
+      <c r="C2" s="36">
         <v>99842</v>
       </c>
-      <c r="D2" s="42">
+      <c r="D2" s="36">
         <v>3</v>
       </c>
-      <c r="E2" s="42">
+      <c r="E2" s="36">
         <f>C2*D2</f>
         <v>299526</v>
       </c>
-      <c r="F2" s="42">
+      <c r="F2" s="36">
         <v>14042</v>
       </c>
-      <c r="G2" s="42">
+      <c r="G2" s="36">
         <f>C2+F2+H2+I2</f>
         <v>115700</v>
       </c>
@@ -2240,26 +2258,26 @@
       </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C3" s="44">
+      <c r="C3" s="37">
         <v>7473</v>
       </c>
-      <c r="D3" s="44">
+      <c r="D3" s="37">
         <v>4</v>
       </c>
-      <c r="E3" s="44">
+      <c r="E3" s="37">
         <f t="shared" ref="E3:E4" si="0">C3*D3</f>
         <v>29892</v>
       </c>
-      <c r="F3" s="44">
+      <c r="F3" s="37">
         <v>1319</v>
       </c>
-      <c r="G3" s="44">
+      <c r="G3" s="37">
         <f>C3+F3</f>
         <v>8792</v>
       </c>
@@ -2271,20 +2289,20 @@
       <c r="B4" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="C4" s="45">
+      <c r="C4" s="38">
         <v>460341</v>
       </c>
-      <c r="D4" s="45">
+      <c r="D4" s="38">
         <v>1</v>
       </c>
-      <c r="E4" s="45">
+      <c r="E4" s="38">
         <f t="shared" si="0"/>
         <v>460341</v>
       </c>
-      <c r="F4" s="45">
+      <c r="F4" s="38">
         <v>24229</v>
       </c>
-      <c r="G4" s="45">
+      <c r="G4" s="38">
         <v>484570</v>
       </c>
     </row>
@@ -2318,54 +2336,54 @@
       <c r="C1" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="D1" s="46" t="s">
+      <c r="D1" s="39" t="s">
+        <v>150</v>
+      </c>
+      <c r="E1" s="39" t="s">
+        <v>151</v>
+      </c>
+      <c r="F1" s="39" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="C2" s="4">
+        <v>420</v>
+      </c>
+      <c r="D2" s="40" t="s">
         <v>142</v>
       </c>
-      <c r="E1" s="46" t="s">
+      <c r="E2" s="40" t="s">
         <v>143</v>
       </c>
-      <c r="F1" s="46" t="s">
+      <c r="F2" s="42" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="43" t="s">
-        <v>138</v>
-      </c>
-      <c r="B2" s="43" t="s">
-        <v>139</v>
-      </c>
-      <c r="C2" s="43">
-        <v>420</v>
-      </c>
-      <c r="D2" s="47">
-        <v>0.2487</v>
-      </c>
-      <c r="E2" s="47">
-        <v>0.23630000000000001</v>
-      </c>
-      <c r="F2" s="49">
-        <v>0</v>
-      </c>
-    </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="C3" s="43">
+      <c r="C3" s="4">
         <v>928</v>
       </c>
-      <c r="D3" s="47">
-        <v>0.2576</v>
-      </c>
-      <c r="E3" s="47">
-        <v>0.28160000000000002</v>
-      </c>
-      <c r="F3" s="47">
-        <v>9.9000000000000008E-3</v>
+      <c r="D3" s="40" t="s">
+        <v>145</v>
+      </c>
+      <c r="E3" s="40" t="s">
+        <v>146</v>
+      </c>
+      <c r="F3" s="40" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -2378,14 +2396,14 @@
       <c r="C4" s="5">
         <v>2868</v>
       </c>
-      <c r="D4" s="48">
-        <v>0.25130000000000002</v>
-      </c>
-      <c r="E4" s="48">
-        <v>0.2329</v>
-      </c>
-      <c r="F4" s="50">
-        <v>0</v>
+      <c r="D4" s="41" t="s">
+        <v>148</v>
+      </c>
+      <c r="E4" s="41" t="s">
+        <v>149</v>
+      </c>
+      <c r="F4" s="43" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>